<commit_message>
Fix data misattribution: Solution-2 decision-log export was filed under Stage 3 but currentSubGoal was never populated in that run
</commit_message>
<xml_diff>
--- a/data/01-fixed-motivation/solution1_records.xlsx
+++ b/data/01-fixed-motivation/solution1_records.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liyihan/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liyihan/dev/ai-town-island-research/data/01-fixed-motivation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5575B16A-7BEF-474D-A51C-93140A6E551C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD3A069-5A00-BF4D-8EA8-EBC4DF8A7275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17000" activeTab="1" xr2:uid="{8391C30E-7080-404D-94AF-F247D6AF26A3}"/>
+    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="16880" activeTab="1" xr2:uid="{8391C30E-7080-404D-94AF-F247D6AF26A3}"/>
   </bookViews>
   <sheets>
-    <sheet name="messages_方案一" sheetId="1" r:id="rId1"/>
-    <sheet name="memories_方案一" sheetId="2" r:id="rId2"/>
+    <sheet name="messages" sheetId="1" r:id="rId1"/>
+    <sheet name="memories" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">messages_方案一!$C$2:$C$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">messages!$C$2:$C$99</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3199,7 +3199,7 @@
         <v>115</v>
       </c>
       <c r="C98" t="str">
-        <f t="shared" ref="C98:C129" si="3">MID(B98,FIND(":",B98)+1,99)</f>
+        <f t="shared" ref="C98:C99" si="3">MID(B98,FIND(":",B98)+1,99)</f>
         <v>3364</v>
       </c>
       <c r="D98" t="s">

</xml_diff>